<commit_message>
test/update Admin test cases
</commit_message>
<xml_diff>
--- a/TestCases_Docs/Admin_Tcs.xlsx
+++ b/TestCases_Docs/Admin_Tcs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FOTOH_COMPU\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1FE57BA-BA4B-4EB5-834C-7D79D9EAE063}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B173F4-A858-4F26-8FE5-611D6DF708D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="832" uniqueCount="378">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -105,9 +105,6 @@
     <t>Hager Elwan</t>
   </si>
   <si>
-    <t>TC-Admin-002</t>
-  </si>
-  <si>
     <t>Verify admin can remove an existing product</t>
   </si>
   <si>
@@ -172,12 +169,6 @@
   </si>
   <si>
     <t>Verify admin can remove an existing supplier</t>
-  </si>
-  <si>
-    <t>1.click customer
-2.Select supplier
-3.Click Remove
-4.Confirm deletion</t>
   </si>
   <si>
     <t>Existing supplier</t>
@@ -255,11 +246,6 @@
   </si>
   <si>
     <t>Missing product name or price</t>
-  </si>
-  <si>
-    <t>Product is not added and validation message
- is displayed
- "please enter the required data"</t>
   </si>
   <si>
     <t>No product is created</t>
@@ -1554,9 +1540,6 @@
 </t>
   </si>
   <si>
-    <t>Open URL, Supplier is logged in</t>
-  </si>
-  <si>
     <t>1.click products 
 2.Select a product status filter 
 3.Check displayed products</t>
@@ -1580,7 +1563,63 @@
     <t>TC-Admin-018</t>
   </si>
   <si>
-    <t>TC-Supplier-019</t>
+    <t>TC-Admin-019</t>
+  </si>
+  <si>
+    <t>Product is not added and validation message
+ is displayed
+ "please enter the valid data"</t>
+  </si>
+  <si>
+    <t>Verify system prevents creating duplicate customer account with same email</t>
+  </si>
+  <si>
+    <t>Open URL, Admin is logged in and a customer account with the same email already exists</t>
+  </si>
+  <si>
+    <t>Existing customer email</t>
+  </si>
+  <si>
+    <t>System shows "Email already exists" message and customer account is not created</t>
+  </si>
+  <si>
+    <t>No duplicate customer account is created</t>
+  </si>
+  <si>
+    <t>1.click on actions section
+ 2.Click Add user
+3.Enter valid Username, existing Email, valid Password, and 4.click on customer radio button
+5.Click Save</t>
+  </si>
+  <si>
+    <t>Verify system prevents creating duplicate supplier account with same email</t>
+  </si>
+  <si>
+    <t>1.click on actions section
+ 2.Click Add user
+3.Enter valid Username, existing Email, valid Password, and 4.click on supplier radio button
+5.Click Save</t>
+  </si>
+  <si>
+    <t>Existing supplier email</t>
+  </si>
+  <si>
+    <t>System shows "Email already exists" message and supplier account is not created</t>
+  </si>
+  <si>
+    <t>1.click supplier
+2.Select supplier
+3.Click Remove
+4.Confirm deletion</t>
+  </si>
+  <si>
+    <t>TC-Admin-017</t>
+  </si>
+  <si>
+    <t>TC-Admin-020</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TC-Admin-002</t>
   </si>
 </sst>
 </file>
@@ -2089,18 +2128,18 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AA976"/>
+  <dimension ref="A1:AA978"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="20" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.08984375" style="39" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.81640625" style="39" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="134.90625" style="39" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.26953125" style="39" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.54296875" style="39" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.26953125" style="39" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.90625" style="39" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="72.54296875" style="39" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="38" style="39" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="76.1796875" style="39" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="47.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="51.36328125" style="39" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.36328125" style="39" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.36328125" style="39" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="23.7265625" style="39" bestFit="1" customWidth="1"/>
@@ -2175,7 +2214,7 @@
         <v>15</v>
       </c>
       <c r="B2" s="38" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="C2" s="38" t="s">
         <v>16</v>
@@ -2191,7 +2230,7 @@
       </c>
       <c r="G2" s="40"/>
       <c r="H2" s="40" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="I2" s="38" t="s">
         <v>20</v>
@@ -2225,33 +2264,33 @@
       <c r="Z2" s="38"/>
       <c r="AA2" s="38"/>
     </row>
-    <row r="3" spans="1:27" ht="105" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" ht="84" x14ac:dyDescent="0.25">
       <c r="A3" s="41" t="s">
-        <v>26</v>
+        <v>377</v>
       </c>
       <c r="B3" s="41" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C3" s="41" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D3" s="41" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E3" s="41" t="s">
         <v>18</v>
       </c>
       <c r="F3" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="G3" s="41" t="s">
+        <v>69</v>
+      </c>
+      <c r="H3" s="42" t="s">
+        <v>363</v>
+      </c>
+      <c r="I3" s="41" t="s">
         <v>70</v>
-      </c>
-      <c r="G3" s="41" t="s">
-        <v>71</v>
-      </c>
-      <c r="H3" s="42" t="s">
-        <v>72</v>
-      </c>
-      <c r="I3" s="41" t="s">
-        <v>73</v>
       </c>
       <c r="J3" s="41" t="s">
         <v>21</v>
@@ -2286,31 +2325,31 @@
     </row>
     <row r="4" spans="1:27" ht="84" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C4" s="38" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E4" s="40" t="s">
         <v>18</v>
       </c>
       <c r="F4" s="40" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="40" t="s">
+      <c r="H4" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="38" t="s">
+      <c r="I4" s="38" t="s">
         <v>31</v>
-      </c>
-      <c r="I4" s="38" t="s">
-        <v>32</v>
       </c>
       <c r="J4" s="41" t="s">
         <v>21</v>
@@ -2319,7 +2358,7 @@
         <v>22</v>
       </c>
       <c r="L4" s="38" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M4" s="38" t="s">
         <v>24</v>
@@ -2341,33 +2380,33 @@
       <c r="Z4" s="38"/>
       <c r="AA4" s="38"/>
     </row>
-    <row r="5" spans="1:27" ht="126" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="38" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B5" s="40" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C5" s="38" t="s">
         <v>16</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E5" s="40" t="s">
         <v>18</v>
       </c>
       <c r="F5" s="40" t="s">
+        <v>312</v>
+      </c>
+      <c r="G5" s="40" t="s">
+        <v>313</v>
+      </c>
+      <c r="H5" s="40" t="s">
         <v>315</v>
       </c>
-      <c r="G5" s="40" t="s">
-        <v>316</v>
-      </c>
-      <c r="H5" s="40" t="s">
-        <v>318</v>
-      </c>
       <c r="I5" s="38" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="J5" s="41" t="s">
         <v>21</v>
@@ -2376,7 +2415,7 @@
         <v>22</v>
       </c>
       <c r="L5" s="38" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M5" s="38" t="s">
         <v>24</v>
@@ -2400,31 +2439,31 @@
     </row>
     <row r="6" spans="1:27" ht="84" x14ac:dyDescent="0.25">
       <c r="A6" s="38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B6" s="40" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6" s="38" t="s">
         <v>16</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E6" s="40" t="s">
         <v>18</v>
       </c>
       <c r="F6" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="G6" s="40" t="s">
+      <c r="H6" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="H6" s="40" t="s">
+      <c r="I6" s="38" t="s">
         <v>40</v>
-      </c>
-      <c r="I6" s="38" t="s">
-        <v>41</v>
       </c>
       <c r="J6" s="41" t="s">
         <v>21</v>
@@ -2433,7 +2472,7 @@
         <v>22</v>
       </c>
       <c r="L6" s="38" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M6" s="38" t="s">
         <v>24</v>
@@ -2457,42 +2496,42 @@
       <c r="Z6" s="38"/>
       <c r="AA6" s="38"/>
     </row>
-    <row r="7" spans="1:27" ht="126" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="C7" s="38" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E7" s="40" t="s">
-        <v>18</v>
+        <v>365</v>
       </c>
       <c r="F7" s="40" t="s">
-        <v>320</v>
+        <v>369</v>
       </c>
       <c r="G7" s="40" t="s">
-        <v>43</v>
+        <v>366</v>
       </c>
       <c r="H7" s="40" t="s">
-        <v>321</v>
-      </c>
-      <c r="I7" s="40" t="s">
-        <v>322</v>
+        <v>367</v>
+      </c>
+      <c r="I7" s="38" t="s">
+        <v>368</v>
       </c>
       <c r="J7" s="41" t="s">
-        <v>21</v>
+        <v>332</v>
       </c>
       <c r="K7" s="38" t="s">
         <v>22</v>
       </c>
       <c r="L7" s="38" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="M7" s="38" t="s">
         <v>24</v>
@@ -2500,9 +2539,7 @@
       <c r="N7" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="O7" s="38" t="s">
-        <v>22</v>
-      </c>
+      <c r="O7" s="38"/>
       <c r="P7" s="38"/>
       <c r="Q7" s="38"/>
       <c r="R7" s="38"/>
@@ -2516,33 +2553,33 @@
       <c r="Z7" s="38"/>
       <c r="AA7" s="38"/>
     </row>
-    <row r="8" spans="1:27" ht="84" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" ht="105" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B8" s="40" t="s">
-        <v>46</v>
+        <v>316</v>
       </c>
       <c r="C8" s="38" t="s">
         <v>16</v>
       </c>
       <c r="D8" s="38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E8" s="40" t="s">
         <v>18</v>
       </c>
       <c r="F8" s="40" t="s">
-        <v>47</v>
+        <v>317</v>
       </c>
       <c r="G8" s="40" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H8" s="40" t="s">
-        <v>49</v>
-      </c>
-      <c r="I8" s="38" t="s">
-        <v>50</v>
+        <v>318</v>
+      </c>
+      <c r="I8" s="40" t="s">
+        <v>319</v>
       </c>
       <c r="J8" s="41" t="s">
         <v>21</v>
@@ -2551,7 +2588,7 @@
         <v>22</v>
       </c>
       <c r="L8" s="38" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="M8" s="38" t="s">
         <v>24</v>
@@ -2575,31 +2612,33 @@
       <c r="Z8" s="38"/>
       <c r="AA8" s="38"/>
     </row>
-    <row r="9" spans="1:27" ht="63" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" ht="84" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
-        <v>55</v>
-      </c>
-      <c r="B9" s="43" t="s">
-        <v>323</v>
+        <v>53</v>
+      </c>
+      <c r="B9" s="40" t="s">
+        <v>45</v>
       </c>
       <c r="C9" s="38" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E9" s="40" t="s">
         <v>18</v>
       </c>
       <c r="F9" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="G9" s="40"/>
+        <v>374</v>
+      </c>
+      <c r="G9" s="40" t="s">
+        <v>46</v>
+      </c>
       <c r="H9" s="40" t="s">
-        <v>324</v>
+        <v>47</v>
       </c>
       <c r="I9" s="38" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="J9" s="41" t="s">
         <v>21</v>
@@ -2608,7 +2647,7 @@
         <v>22</v>
       </c>
       <c r="L9" s="38" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="M9" s="38" t="s">
         <v>24</v>
@@ -2634,38 +2673,40 @@
     </row>
     <row r="10" spans="1:27" ht="105" x14ac:dyDescent="0.25">
       <c r="A10" s="38" t="s">
-        <v>56</v>
-      </c>
-      <c r="B10" s="43" t="s">
-        <v>325</v>
+        <v>54</v>
+      </c>
+      <c r="B10" s="40" t="s">
+        <v>370</v>
       </c>
       <c r="C10" s="38" t="s">
         <v>16</v>
       </c>
       <c r="D10" s="38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E10" s="40" t="s">
-        <v>18</v>
+        <v>365</v>
       </c>
       <c r="F10" s="40" t="s">
-        <v>330</v>
-      </c>
-      <c r="G10" s="40"/>
+        <v>371</v>
+      </c>
+      <c r="G10" s="40" t="s">
+        <v>372</v>
+      </c>
       <c r="H10" s="40" t="s">
-        <v>326</v>
+        <v>373</v>
       </c>
       <c r="I10" s="38" t="s">
-        <v>53</v>
+        <v>368</v>
       </c>
       <c r="J10" s="41" t="s">
-        <v>21</v>
+        <v>332</v>
       </c>
       <c r="K10" s="38" t="s">
         <v>22</v>
       </c>
       <c r="L10" s="38" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="M10" s="38" t="s">
         <v>24</v>
@@ -2673,9 +2714,7 @@
       <c r="N10" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="O10" s="38" t="s">
-        <v>22</v>
-      </c>
+      <c r="O10" s="38"/>
       <c r="P10" s="38"/>
       <c r="Q10" s="38"/>
       <c r="R10" s="38"/>
@@ -2689,31 +2728,31 @@
       <c r="Z10" s="38"/>
       <c r="AA10" s="38"/>
     </row>
-    <row r="11" spans="1:27" ht="105" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" ht="63" x14ac:dyDescent="0.25">
       <c r="A11" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B11" s="40" t="s">
-        <v>327</v>
+        <v>56</v>
+      </c>
+      <c r="B11" s="43" t="s">
+        <v>320</v>
       </c>
       <c r="C11" s="38" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E11" s="40" t="s">
         <v>18</v>
       </c>
       <c r="F11" s="40" t="s">
-        <v>329</v>
+        <v>50</v>
       </c>
       <c r="G11" s="40"/>
       <c r="H11" s="40" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="J11" s="41" t="s">
         <v>21</v>
@@ -2722,7 +2761,7 @@
         <v>22</v>
       </c>
       <c r="L11" s="38" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="M11" s="38" t="s">
         <v>24</v>
@@ -2747,159 +2786,155 @@
       <c r="AA11" s="38"/>
     </row>
     <row r="12" spans="1:27" ht="84" x14ac:dyDescent="0.25">
-      <c r="A12" s="41" t="s">
-        <v>63</v>
-      </c>
-      <c r="B12" s="41" t="s">
-        <v>313</v>
-      </c>
-      <c r="C12" s="41" t="s">
+      <c r="A12" s="38" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="43" t="s">
+        <v>322</v>
+      </c>
+      <c r="C12" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12" s="41" t="s">
+      <c r="D12" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="F12" s="42" t="s">
-        <v>310</v>
-      </c>
-      <c r="G12" s="41" t="s">
-        <v>59</v>
-      </c>
-      <c r="H12" s="41" t="s">
-        <v>60</v>
-      </c>
-      <c r="I12" s="41" t="s">
-        <v>61</v>
+      <c r="F12" s="40" t="s">
+        <v>327</v>
+      </c>
+      <c r="G12" s="40"/>
+      <c r="H12" s="40" t="s">
+        <v>323</v>
+      </c>
+      <c r="I12" s="38" t="s">
+        <v>51</v>
       </c>
       <c r="J12" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="K12" s="41" t="s">
+      <c r="K12" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="L12" s="41" t="s">
-        <v>62</v>
-      </c>
-      <c r="M12" s="41" t="s">
+      <c r="L12" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="M12" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="N12" s="41" t="s">
+      <c r="N12" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="O12" s="41" t="s">
+      <c r="O12" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="P12" s="41"/>
-      <c r="Q12" s="41"/>
-      <c r="R12" s="41"/>
-      <c r="S12" s="41"/>
-      <c r="T12" s="41"/>
-      <c r="U12" s="41"/>
-      <c r="V12" s="41"/>
-      <c r="W12" s="41"/>
-      <c r="X12" s="41"/>
-      <c r="Y12" s="41"/>
-      <c r="Z12" s="41"/>
-      <c r="AA12" s="41"/>
+      <c r="P12" s="38"/>
+      <c r="Q12" s="38"/>
+      <c r="R12" s="38"/>
+      <c r="S12" s="38"/>
+      <c r="T12" s="38"/>
+      <c r="U12" s="38"/>
+      <c r="V12" s="38"/>
+      <c r="W12" s="38"/>
+      <c r="X12" s="38"/>
+      <c r="Y12" s="38"/>
+      <c r="Z12" s="38"/>
+      <c r="AA12" s="38"/>
     </row>
     <row r="13" spans="1:27" ht="84" x14ac:dyDescent="0.25">
-      <c r="A13" s="41" t="s">
-        <v>67</v>
-      </c>
-      <c r="B13" s="41" t="s">
-        <v>64</v>
-      </c>
-      <c r="C13" s="41" t="s">
+      <c r="A13" s="38" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" s="40" t="s">
+        <v>324</v>
+      </c>
+      <c r="C13" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="E13" s="41" t="s">
+      <c r="D13" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="42" t="s">
-        <v>311</v>
-      </c>
-      <c r="G13" s="41" t="s">
-        <v>59</v>
-      </c>
-      <c r="H13" s="41" t="s">
-        <v>65</v>
-      </c>
-      <c r="I13" s="41" t="s">
-        <v>66</v>
+      <c r="F13" s="40" t="s">
+        <v>326</v>
+      </c>
+      <c r="G13" s="40"/>
+      <c r="H13" s="40" t="s">
+        <v>325</v>
+      </c>
+      <c r="I13" s="38" t="s">
+        <v>51</v>
       </c>
       <c r="J13" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="K13" s="41" t="s">
+      <c r="K13" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="L13" s="41" t="s">
-        <v>62</v>
-      </c>
-      <c r="M13" s="41" t="s">
+      <c r="L13" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="M13" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="N13" s="41" t="s">
+      <c r="N13" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="O13" s="41" t="s">
+      <c r="O13" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="P13" s="41"/>
-      <c r="Q13" s="41"/>
-      <c r="R13" s="41"/>
-      <c r="S13" s="41"/>
-      <c r="T13" s="41"/>
-      <c r="U13" s="41"/>
-      <c r="V13" s="41"/>
-      <c r="W13" s="41"/>
-      <c r="X13" s="41"/>
-      <c r="Y13" s="41"/>
-      <c r="Z13" s="41"/>
-      <c r="AA13" s="41"/>
-    </row>
-    <row r="14" spans="1:27" ht="63" x14ac:dyDescent="0.25">
+      <c r="P13" s="38"/>
+      <c r="Q13" s="38"/>
+      <c r="R13" s="38"/>
+      <c r="S13" s="38"/>
+      <c r="T13" s="38"/>
+      <c r="U13" s="38"/>
+      <c r="V13" s="38"/>
+      <c r="W13" s="38"/>
+      <c r="X13" s="38"/>
+      <c r="Y13" s="38"/>
+      <c r="Z13" s="38"/>
+      <c r="AA13" s="38"/>
+    </row>
+    <row r="14" spans="1:27" ht="84" x14ac:dyDescent="0.25">
       <c r="A14" s="41" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B14" s="41" t="s">
-        <v>332</v>
+        <v>310</v>
       </c>
       <c r="C14" s="41" t="s">
         <v>16</v>
       </c>
       <c r="D14" s="41" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E14" s="41" t="s">
         <v>18</v>
       </c>
       <c r="F14" s="42" t="s">
-        <v>336</v>
+        <v>307</v>
       </c>
       <c r="G14" s="41" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="H14" s="41" t="s">
-        <v>333</v>
+        <v>58</v>
       </c>
       <c r="I14" s="41" t="s">
-        <v>334</v>
+        <v>59</v>
       </c>
       <c r="J14" s="41" t="s">
-        <v>335</v>
+        <v>21</v>
       </c>
       <c r="K14" s="41" t="s">
         <v>22</v>
       </c>
       <c r="L14" s="41" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M14" s="41" t="s">
         <v>24</v>
@@ -2907,7 +2942,9 @@
       <c r="N14" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="O14" s="41"/>
+      <c r="O14" s="41" t="s">
+        <v>22</v>
+      </c>
       <c r="P14" s="41"/>
       <c r="Q14" s="41"/>
       <c r="R14" s="41"/>
@@ -2921,156 +2958,158 @@
       <c r="Z14" s="41"/>
       <c r="AA14" s="41"/>
     </row>
-    <row r="15" spans="1:27" ht="105" x14ac:dyDescent="0.25">
-      <c r="A15" s="38" t="s">
-        <v>75</v>
-      </c>
-      <c r="B15" s="38" t="s">
-        <v>337</v>
-      </c>
-      <c r="C15" s="38" t="s">
+    <row r="15" spans="1:27" ht="84" x14ac:dyDescent="0.25">
+      <c r="A15" s="41" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="38" t="s">
-        <v>28</v>
-      </c>
-      <c r="E15" s="38" t="s">
-        <v>338</v>
-      </c>
-      <c r="F15" s="40" t="s">
-        <v>339</v>
-      </c>
-      <c r="G15" s="38" t="s">
+      <c r="D15" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="42" t="s">
+        <v>308</v>
+      </c>
+      <c r="G15" s="41" t="s">
+        <v>57</v>
+      </c>
+      <c r="H15" s="41" t="s">
+        <v>63</v>
+      </c>
+      <c r="I15" s="41" t="s">
+        <v>64</v>
+      </c>
+      <c r="J15" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="K15" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="H15" s="40" t="s">
-        <v>340</v>
-      </c>
-      <c r="I15" s="38" t="s">
-        <v>341</v>
-      </c>
-      <c r="J15" s="38" t="s">
-        <v>335</v>
-      </c>
-      <c r="K15" s="38" t="s">
+      <c r="L15" s="41" t="s">
+        <v>60</v>
+      </c>
+      <c r="M15" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="N15" s="41" t="s">
+        <v>25</v>
+      </c>
+      <c r="O15" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="L15" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="M15" s="38" t="s">
+      <c r="P15" s="41"/>
+      <c r="Q15" s="41"/>
+      <c r="R15" s="41"/>
+      <c r="S15" s="41"/>
+      <c r="T15" s="41"/>
+      <c r="U15" s="41"/>
+      <c r="V15" s="41"/>
+      <c r="W15" s="41"/>
+      <c r="X15" s="41"/>
+      <c r="Y15" s="41"/>
+      <c r="Z15" s="41"/>
+      <c r="AA15" s="41"/>
+    </row>
+    <row r="16" spans="1:27" ht="42" x14ac:dyDescent="0.25">
+      <c r="A16" s="41" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="41" t="s">
+        <v>329</v>
+      </c>
+      <c r="C16" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="42" t="s">
+        <v>333</v>
+      </c>
+      <c r="G16" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="H16" s="41" t="s">
+        <v>330</v>
+      </c>
+      <c r="I16" s="41" t="s">
+        <v>331</v>
+      </c>
+      <c r="J16" s="41" t="s">
+        <v>332</v>
+      </c>
+      <c r="K16" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="L16" s="41" t="s">
+        <v>60</v>
+      </c>
+      <c r="M16" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="N15" s="38" t="s">
+      <c r="N16" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="O15" s="38"/>
-      <c r="P15" s="38"/>
-      <c r="Q15" s="38"/>
-      <c r="R15" s="38"/>
-      <c r="S15" s="38"/>
-      <c r="T15" s="38"/>
-      <c r="U15" s="38"/>
-      <c r="V15" s="38"/>
-      <c r="W15" s="38"/>
-      <c r="X15" s="38"/>
-      <c r="Y15" s="38"/>
-      <c r="Z15" s="38"/>
-      <c r="AA15" s="38"/>
-    </row>
-    <row r="16" spans="1:27" ht="105" x14ac:dyDescent="0.25">
-      <c r="A16" s="38" t="s">
-        <v>76</v>
-      </c>
-      <c r="B16" s="38" t="s">
-        <v>342</v>
-      </c>
-      <c r="C16" s="38" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" s="38" t="s">
-        <v>28</v>
-      </c>
-      <c r="E16" s="38" t="s">
-        <v>338</v>
-      </c>
-      <c r="F16" s="40" t="s">
-        <v>345</v>
-      </c>
-      <c r="G16" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="H16" s="38" t="s">
-        <v>343</v>
-      </c>
-      <c r="I16" s="38" t="s">
-        <v>344</v>
-      </c>
-      <c r="J16" s="38" t="s">
-        <v>335</v>
-      </c>
-      <c r="K16" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="L16" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="M16" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="N16" s="38" t="s">
-        <v>25</v>
-      </c>
-      <c r="O16" s="38"/>
-      <c r="P16" s="38"/>
-      <c r="Q16" s="38"/>
-      <c r="R16" s="38"/>
-      <c r="S16" s="38"/>
-      <c r="T16" s="38"/>
-      <c r="U16" s="38"/>
-      <c r="V16" s="38"/>
-      <c r="W16" s="38"/>
-      <c r="X16" s="38"/>
-      <c r="Y16" s="38"/>
-      <c r="Z16" s="38"/>
-      <c r="AA16" s="38"/>
-    </row>
-    <row r="17" spans="1:27" ht="63" x14ac:dyDescent="0.25">
+      <c r="O16" s="41"/>
+      <c r="P16" s="41"/>
+      <c r="Q16" s="41"/>
+      <c r="R16" s="41"/>
+      <c r="S16" s="41"/>
+      <c r="T16" s="41"/>
+      <c r="U16" s="41"/>
+      <c r="V16" s="41"/>
+      <c r="W16" s="41"/>
+      <c r="X16" s="41"/>
+      <c r="Y16" s="41"/>
+      <c r="Z16" s="41"/>
+      <c r="AA16" s="41"/>
+    </row>
+    <row r="17" spans="1:27" ht="84" x14ac:dyDescent="0.25">
       <c r="A17" s="38" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="B17" s="38" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="C17" s="38" t="s">
         <v>16</v>
       </c>
       <c r="D17" s="38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>351</v>
+        <v>335</v>
       </c>
       <c r="F17" s="40" t="s">
-        <v>352</v>
+        <v>336</v>
       </c>
       <c r="G17" s="38" t="s">
-        <v>347</v>
-      </c>
-      <c r="H17" s="38" t="s">
-        <v>348</v>
+        <v>22</v>
+      </c>
+      <c r="H17" s="40" t="s">
+        <v>337</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="J17" s="38" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="K17" s="38" t="s">
         <v>22</v>
       </c>
       <c r="L17" s="38" t="s">
-        <v>350</v>
+        <v>60</v>
       </c>
       <c r="M17" s="38" t="s">
         <v>24</v>
@@ -3092,42 +3131,42 @@
       <c r="Z17" s="38"/>
       <c r="AA17" s="38"/>
     </row>
-    <row r="18" spans="1:27" ht="105" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:27" ht="84" x14ac:dyDescent="0.25">
       <c r="A18" s="38" t="s">
-        <v>365</v>
+        <v>375</v>
       </c>
       <c r="B18" s="38" t="s">
-        <v>353</v>
+        <v>339</v>
       </c>
       <c r="C18" s="38" t="s">
         <v>16</v>
       </c>
       <c r="D18" s="38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E18" s="38" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="F18" s="40" t="s">
-        <v>357</v>
+        <v>342</v>
       </c>
       <c r="G18" s="38" t="s">
-        <v>354</v>
+        <v>22</v>
       </c>
       <c r="H18" s="38" t="s">
-        <v>355</v>
+        <v>340</v>
       </c>
       <c r="I18" s="38" t="s">
-        <v>356</v>
+        <v>341</v>
       </c>
       <c r="J18" s="38" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="K18" s="38" t="s">
         <v>22</v>
       </c>
       <c r="L18" s="38" t="s">
-        <v>350</v>
+        <v>60</v>
       </c>
       <c r="M18" s="38" t="s">
         <v>24</v>
@@ -3151,40 +3190,40 @@
     </row>
     <row r="19" spans="1:27" ht="63" x14ac:dyDescent="0.25">
       <c r="A19" s="38" t="s">
-        <v>366</v>
-      </c>
-      <c r="B19" s="40" t="s">
-        <v>362</v>
+        <v>361</v>
+      </c>
+      <c r="B19" s="38" t="s">
+        <v>343</v>
       </c>
       <c r="C19" s="38" t="s">
         <v>16</v>
       </c>
       <c r="D19" s="38" t="s">
-        <v>28</v>
-      </c>
-      <c r="E19" s="40" t="s">
-        <v>358</v>
+        <v>27</v>
+      </c>
+      <c r="E19" s="38" t="s">
+        <v>348</v>
       </c>
       <c r="F19" s="40" t="s">
-        <v>359</v>
-      </c>
-      <c r="G19" s="40" t="s">
-        <v>22</v>
-      </c>
-      <c r="H19" s="40" t="s">
-        <v>360</v>
-      </c>
-      <c r="I19" s="40" t="s">
-        <v>361</v>
-      </c>
-      <c r="J19" s="41" t="s">
-        <v>335</v>
+        <v>349</v>
+      </c>
+      <c r="G19" s="38" t="s">
+        <v>344</v>
+      </c>
+      <c r="H19" s="38" t="s">
+        <v>345</v>
+      </c>
+      <c r="I19" s="38" t="s">
+        <v>346</v>
+      </c>
+      <c r="J19" s="38" t="s">
+        <v>332</v>
       </c>
       <c r="K19" s="38" t="s">
         <v>22</v>
       </c>
       <c r="L19" s="38" t="s">
-        <v>363</v>
+        <v>347</v>
       </c>
       <c r="M19" s="38" t="s">
         <v>24</v>
@@ -3206,21 +3245,49 @@
       <c r="Z19" s="38"/>
       <c r="AA19" s="38"/>
     </row>
-    <row r="20" spans="1:27" ht="21" x14ac:dyDescent="0.25">
-      <c r="A20" s="38"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="40"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="40"/>
-      <c r="H20" s="40"/>
-      <c r="I20" s="38"/>
-      <c r="J20" s="38"/>
-      <c r="K20" s="38"/>
-      <c r="L20" s="38"/>
-      <c r="M20" s="38"/>
-      <c r="N20" s="38"/>
+    <row r="20" spans="1:27" ht="84" x14ac:dyDescent="0.25">
+      <c r="A20" s="38" t="s">
+        <v>362</v>
+      </c>
+      <c r="B20" s="38" t="s">
+        <v>350</v>
+      </c>
+      <c r="C20" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="38" t="s">
+        <v>335</v>
+      </c>
+      <c r="F20" s="40" t="s">
+        <v>354</v>
+      </c>
+      <c r="G20" s="38" t="s">
+        <v>351</v>
+      </c>
+      <c r="H20" s="38" t="s">
+        <v>352</v>
+      </c>
+      <c r="I20" s="38" t="s">
+        <v>353</v>
+      </c>
+      <c r="J20" s="38" t="s">
+        <v>332</v>
+      </c>
+      <c r="K20" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="L20" s="38" t="s">
+        <v>347</v>
+      </c>
+      <c r="M20" s="38" t="s">
+        <v>24</v>
+      </c>
+      <c r="N20" s="38" t="s">
+        <v>25</v>
+      </c>
       <c r="O20" s="38"/>
       <c r="P20" s="38"/>
       <c r="Q20" s="38"/>
@@ -3235,21 +3302,49 @@
       <c r="Z20" s="38"/>
       <c r="AA20" s="38"/>
     </row>
-    <row r="21" spans="1:27" ht="21" x14ac:dyDescent="0.25">
-      <c r="A21" s="38"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="38"/>
-      <c r="J21" s="38"/>
-      <c r="K21" s="38"/>
-      <c r="L21" s="38"/>
-      <c r="M21" s="38"/>
-      <c r="N21" s="38"/>
+    <row r="21" spans="1:27" ht="63" x14ac:dyDescent="0.25">
+      <c r="A21" s="38" t="s">
+        <v>376</v>
+      </c>
+      <c r="B21" s="40" t="s">
+        <v>358</v>
+      </c>
+      <c r="C21" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="40" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" s="40" t="s">
+        <v>355</v>
+      </c>
+      <c r="G21" s="40" t="s">
+        <v>22</v>
+      </c>
+      <c r="H21" s="40" t="s">
+        <v>356</v>
+      </c>
+      <c r="I21" s="40" t="s">
+        <v>357</v>
+      </c>
+      <c r="J21" s="41" t="s">
+        <v>332</v>
+      </c>
+      <c r="K21" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="L21" s="38" t="s">
+        <v>359</v>
+      </c>
+      <c r="M21" s="38" t="s">
+        <v>24</v>
+      </c>
+      <c r="N21" s="38" t="s">
+        <v>25</v>
+      </c>
       <c r="O21" s="38"/>
       <c r="P21" s="38"/>
       <c r="Q21" s="38"/>
@@ -3271,7 +3366,7 @@
       <c r="D22" s="38"/>
       <c r="E22" s="40"/>
       <c r="F22" s="40"/>
-      <c r="G22" s="38"/>
+      <c r="G22" s="40"/>
       <c r="H22" s="40"/>
       <c r="I22" s="38"/>
       <c r="J22" s="38"/>
@@ -3300,8 +3395,8 @@
       <c r="D23" s="38"/>
       <c r="E23" s="40"/>
       <c r="F23" s="40"/>
-      <c r="G23" s="38"/>
-      <c r="H23" s="38"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="40"/>
       <c r="I23" s="38"/>
       <c r="J23" s="38"/>
       <c r="K23" s="38"/>
@@ -3330,7 +3425,7 @@
       <c r="E24" s="40"/>
       <c r="F24" s="40"/>
       <c r="G24" s="38"/>
-      <c r="H24" s="38"/>
+      <c r="H24" s="40"/>
       <c r="I24" s="38"/>
       <c r="J24" s="38"/>
       <c r="K24" s="38"/>
@@ -3356,8 +3451,8 @@
       <c r="B25" s="38"/>
       <c r="C25" s="38"/>
       <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="38"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
       <c r="G25" s="38"/>
       <c r="H25" s="38"/>
       <c r="I25" s="38"/>
@@ -3385,8 +3480,8 @@
       <c r="B26" s="38"/>
       <c r="C26" s="38"/>
       <c r="D26" s="38"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="38"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
       <c r="G26" s="38"/>
       <c r="H26" s="38"/>
       <c r="I26" s="38"/>
@@ -3533,7 +3628,7 @@
       <c r="E31" s="38"/>
       <c r="F31" s="38"/>
       <c r="G31" s="38"/>
-      <c r="H31" s="40"/>
+      <c r="H31" s="38"/>
       <c r="I31" s="38"/>
       <c r="J31" s="38"/>
       <c r="K31" s="38"/>
@@ -3591,7 +3686,7 @@
       <c r="E33" s="38"/>
       <c r="F33" s="38"/>
       <c r="G33" s="38"/>
-      <c r="H33" s="38"/>
+      <c r="H33" s="40"/>
       <c r="I33" s="38"/>
       <c r="J33" s="38"/>
       <c r="K33" s="38"/>
@@ -3646,10 +3741,10 @@
       <c r="B35" s="38"/>
       <c r="C35" s="38"/>
       <c r="D35" s="38"/>
-      <c r="E35" s="40"/>
+      <c r="E35" s="38"/>
       <c r="F35" s="38"/>
       <c r="G35" s="38"/>
-      <c r="H35" s="40"/>
+      <c r="H35" s="38"/>
       <c r="I35" s="38"/>
       <c r="J35" s="38"/>
       <c r="K35" s="38"/>
@@ -3675,10 +3770,10 @@
       <c r="B36" s="38"/>
       <c r="C36" s="38"/>
       <c r="D36" s="38"/>
-      <c r="E36" s="40"/>
+      <c r="E36" s="38"/>
       <c r="F36" s="38"/>
       <c r="G36" s="38"/>
-      <c r="H36" s="40"/>
+      <c r="H36" s="38"/>
       <c r="I36" s="38"/>
       <c r="J36" s="38"/>
       <c r="K36" s="38"/>
@@ -3704,10 +3799,10 @@
       <c r="B37" s="38"/>
       <c r="C37" s="38"/>
       <c r="D37" s="38"/>
-      <c r="E37" s="38"/>
+      <c r="E37" s="40"/>
       <c r="F37" s="38"/>
       <c r="G37" s="38"/>
-      <c r="H37" s="38"/>
+      <c r="H37" s="40"/>
       <c r="I37" s="38"/>
       <c r="J37" s="38"/>
       <c r="K37" s="38"/>
@@ -3733,10 +3828,10 @@
       <c r="B38" s="38"/>
       <c r="C38" s="38"/>
       <c r="D38" s="38"/>
-      <c r="E38" s="38"/>
+      <c r="E38" s="40"/>
       <c r="F38" s="38"/>
       <c r="G38" s="38"/>
-      <c r="H38" s="38"/>
+      <c r="H38" s="40"/>
       <c r="I38" s="38"/>
       <c r="J38" s="38"/>
       <c r="K38" s="38"/>
@@ -3760,9 +3855,7 @@
     <row r="39" spans="1:27" ht="21" x14ac:dyDescent="0.25">
       <c r="A39" s="38"/>
       <c r="B39" s="38"/>
-      <c r="C39" s="38" t="s">
-        <v>69</v>
-      </c>
+      <c r="C39" s="38"/>
       <c r="D39" s="38"/>
       <c r="E39" s="38"/>
       <c r="F39" s="38"/>
@@ -3820,7 +3913,9 @@
     <row r="41" spans="1:27" ht="21" x14ac:dyDescent="0.25">
       <c r="A41" s="38"/>
       <c r="B41" s="38"/>
-      <c r="C41" s="38"/>
+      <c r="C41" s="38" t="s">
+        <v>67</v>
+      </c>
       <c r="D41" s="38"/>
       <c r="E41" s="38"/>
       <c r="F41" s="38"/>
@@ -3905,33 +4000,33 @@
       <c r="AA43" s="38"/>
     </row>
     <row r="44" spans="1:27" ht="21" x14ac:dyDescent="0.25">
-      <c r="A44" s="44"/>
-      <c r="B44" s="44"/>
-      <c r="C44" s="44"/>
-      <c r="D44" s="44"/>
-      <c r="E44" s="44"/>
-      <c r="F44" s="44"/>
-      <c r="G44" s="44"/>
-      <c r="H44" s="44"/>
-      <c r="I44" s="44"/>
-      <c r="J44" s="44"/>
-      <c r="K44" s="44"/>
-      <c r="L44" s="44"/>
-      <c r="M44" s="44"/>
-      <c r="N44" s="44"/>
-      <c r="O44" s="44"/>
-      <c r="P44" s="44"/>
-      <c r="Q44" s="44"/>
-      <c r="R44" s="44"/>
-      <c r="S44" s="44"/>
-      <c r="T44" s="44"/>
-      <c r="U44" s="44"/>
-      <c r="V44" s="44"/>
-      <c r="W44" s="44"/>
-      <c r="X44" s="44"/>
-      <c r="Y44" s="44"/>
-      <c r="Z44" s="44"/>
-      <c r="AA44" s="44"/>
+      <c r="A44" s="38"/>
+      <c r="B44" s="38"/>
+      <c r="C44" s="38"/>
+      <c r="D44" s="38"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="38"/>
+      <c r="G44" s="38"/>
+      <c r="H44" s="38"/>
+      <c r="I44" s="38"/>
+      <c r="J44" s="38"/>
+      <c r="K44" s="38"/>
+      <c r="L44" s="38"/>
+      <c r="M44" s="38"/>
+      <c r="N44" s="38"/>
+      <c r="O44" s="38"/>
+      <c r="P44" s="38"/>
+      <c r="Q44" s="38"/>
+      <c r="R44" s="38"/>
+      <c r="S44" s="38"/>
+      <c r="T44" s="38"/>
+      <c r="U44" s="38"/>
+      <c r="V44" s="38"/>
+      <c r="W44" s="38"/>
+      <c r="X44" s="38"/>
+      <c r="Y44" s="38"/>
+      <c r="Z44" s="38"/>
+      <c r="AA44" s="38"/>
     </row>
     <row r="45" spans="1:27" ht="21" x14ac:dyDescent="0.25">
       <c r="A45" s="38"/>
@@ -3963,33 +4058,33 @@
       <c r="AA45" s="38"/>
     </row>
     <row r="46" spans="1:27" ht="21" x14ac:dyDescent="0.25">
-      <c r="A46" s="38"/>
-      <c r="B46" s="38"/>
-      <c r="C46" s="38"/>
-      <c r="D46" s="38"/>
-      <c r="E46" s="38"/>
-      <c r="F46" s="38"/>
-      <c r="G46" s="38"/>
-      <c r="H46" s="38"/>
-      <c r="I46" s="38"/>
-      <c r="J46" s="38"/>
-      <c r="K46" s="38"/>
-      <c r="L46" s="38"/>
-      <c r="M46" s="38"/>
-      <c r="N46" s="38"/>
-      <c r="O46" s="38"/>
-      <c r="P46" s="38"/>
-      <c r="Q46" s="38"/>
-      <c r="R46" s="38"/>
-      <c r="S46" s="38"/>
-      <c r="T46" s="38"/>
-      <c r="U46" s="38"/>
-      <c r="V46" s="38"/>
-      <c r="W46" s="38"/>
-      <c r="X46" s="38"/>
-      <c r="Y46" s="38"/>
-      <c r="Z46" s="38"/>
-      <c r="AA46" s="38"/>
+      <c r="A46" s="44"/>
+      <c r="B46" s="44"/>
+      <c r="C46" s="44"/>
+      <c r="D46" s="44"/>
+      <c r="E46" s="44"/>
+      <c r="F46" s="44"/>
+      <c r="G46" s="44"/>
+      <c r="H46" s="44"/>
+      <c r="I46" s="44"/>
+      <c r="J46" s="44"/>
+      <c r="K46" s="44"/>
+      <c r="L46" s="44"/>
+      <c r="M46" s="44"/>
+      <c r="N46" s="44"/>
+      <c r="O46" s="44"/>
+      <c r="P46" s="44"/>
+      <c r="Q46" s="44"/>
+      <c r="R46" s="44"/>
+      <c r="S46" s="44"/>
+      <c r="T46" s="44"/>
+      <c r="U46" s="44"/>
+      <c r="V46" s="44"/>
+      <c r="W46" s="44"/>
+      <c r="X46" s="44"/>
+      <c r="Y46" s="44"/>
+      <c r="Z46" s="44"/>
+      <c r="AA46" s="44"/>
     </row>
     <row r="47" spans="1:27" ht="21" x14ac:dyDescent="0.25">
       <c r="A47" s="38"/>
@@ -4200,9 +4295,7 @@
       <c r="C54" s="38"/>
       <c r="D54" s="38"/>
       <c r="E54" s="38"/>
-      <c r="F54" s="38" t="s">
-        <v>77</v>
-      </c>
+      <c r="F54" s="38"/>
       <c r="G54" s="38"/>
       <c r="H54" s="38"/>
       <c r="I54" s="38"/>
@@ -4260,7 +4353,9 @@
       <c r="C56" s="38"/>
       <c r="D56" s="38"/>
       <c r="E56" s="38"/>
-      <c r="F56" s="38"/>
+      <c r="F56" s="38" t="s">
+        <v>74</v>
+      </c>
       <c r="G56" s="38"/>
       <c r="H56" s="38"/>
       <c r="I56" s="38"/>
@@ -30963,12 +31058,70 @@
       <c r="Z976" s="38"/>
       <c r="AA976" s="38"/>
     </row>
+    <row r="977" spans="1:27" ht="21" x14ac:dyDescent="0.25">
+      <c r="A977" s="38"/>
+      <c r="B977" s="38"/>
+      <c r="C977" s="38"/>
+      <c r="D977" s="38"/>
+      <c r="E977" s="38"/>
+      <c r="F977" s="38"/>
+      <c r="G977" s="38"/>
+      <c r="H977" s="38"/>
+      <c r="I977" s="38"/>
+      <c r="J977" s="38"/>
+      <c r="K977" s="38"/>
+      <c r="L977" s="38"/>
+      <c r="M977" s="38"/>
+      <c r="N977" s="38"/>
+      <c r="O977" s="38"/>
+      <c r="P977" s="38"/>
+      <c r="Q977" s="38"/>
+      <c r="R977" s="38"/>
+      <c r="S977" s="38"/>
+      <c r="T977" s="38"/>
+      <c r="U977" s="38"/>
+      <c r="V977" s="38"/>
+      <c r="W977" s="38"/>
+      <c r="X977" s="38"/>
+      <c r="Y977" s="38"/>
+      <c r="Z977" s="38"/>
+      <c r="AA977" s="38"/>
+    </row>
+    <row r="978" spans="1:27" ht="21" x14ac:dyDescent="0.25">
+      <c r="A978" s="38"/>
+      <c r="B978" s="38"/>
+      <c r="C978" s="38"/>
+      <c r="D978" s="38"/>
+      <c r="E978" s="38"/>
+      <c r="F978" s="38"/>
+      <c r="G978" s="38"/>
+      <c r="H978" s="38"/>
+      <c r="I978" s="38"/>
+      <c r="J978" s="38"/>
+      <c r="K978" s="38"/>
+      <c r="L978" s="38"/>
+      <c r="M978" s="38"/>
+      <c r="N978" s="38"/>
+      <c r="O978" s="38"/>
+      <c r="P978" s="38"/>
+      <c r="Q978" s="38"/>
+      <c r="R978" s="38"/>
+      <c r="S978" s="38"/>
+      <c r="T978" s="38"/>
+      <c r="U978" s="38"/>
+      <c r="V978" s="38"/>
+      <c r="W978" s="38"/>
+      <c r="X978" s="38"/>
+      <c r="Y978" s="38"/>
+      <c r="Z978" s="38"/>
+      <c r="AA978" s="38"/>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C39:C95 C2:C37" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C41:C97 C2:C39" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"valid,invalid"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J39:J60 J2:J37" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J41:J62 J2:J39" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"in progress,in review,approved,cancelled"</formula1>
     </dataValidation>
   </dataValidations>
@@ -31011,7 +31164,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -31026,7 +31179,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
@@ -31050,54 +31203,54 @@
         <v>14</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:29" ht="99" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="H2" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>88</v>
       </c>
       <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L2" s="3"/>
       <c r="M2" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="P2" s="3"/>
       <c r="Q2" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="R2" s="3"/>
       <c r="S2" s="3"/>
@@ -31114,49 +31267,49 @@
     </row>
     <row r="3" spans="1:29" ht="50" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="G3" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E3" s="5" t="s">
+      <c r="H3" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>99</v>
-      </c>
       <c r="I3" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J3" s="3"/>
       <c r="K3" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="P3" s="3"/>
       <c r="Q3" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="R3" s="3"/>
       <c r="S3" s="3"/>
@@ -31173,49 +31326,49 @@
     </row>
     <row r="4" spans="1:29" ht="100" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>104</v>
-      </c>
       <c r="H4" s="4" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J4" s="3"/>
       <c r="K4" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L4" s="3"/>
       <c r="M4" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -31232,49 +31385,49 @@
     </row>
     <row r="5" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E5" s="5" t="s">
+      <c r="H5" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>110</v>
-      </c>
       <c r="I5" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J5" s="3"/>
       <c r="K5" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L5" s="3"/>
       <c r="M5" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -31291,49 +31444,49 @@
     </row>
     <row r="6" spans="1:29" ht="100" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>114</v>
-      </c>
       <c r="H6" s="7" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J6" s="6"/>
       <c r="K6" s="6" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L6" s="6"/>
       <c r="M6" s="6" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="P6" s="6"/>
       <c r="Q6" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -31350,49 +31503,49 @@
     </row>
     <row r="7" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="H7" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>119</v>
-      </c>
       <c r="I7" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L7" s="3"/>
       <c r="M7" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="P7" s="3"/>
       <c r="Q7" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
@@ -31409,49 +31562,49 @@
     </row>
     <row r="8" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="H8" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>124</v>
-      </c>
       <c r="I8" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J8" s="3"/>
       <c r="K8" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L8" s="3"/>
       <c r="M8" s="3" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="P8" s="3"/>
       <c r="Q8" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
@@ -31468,49 +31621,49 @@
     </row>
     <row r="9" spans="1:29" ht="87.5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E9" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="H9" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="F9" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>131</v>
-      </c>
       <c r="I9" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J9" s="10"/>
       <c r="K9" s="10" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L9" s="10"/>
       <c r="M9" s="6" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="N9" s="10" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="P9" s="10"/>
       <c r="Q9" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="R9" s="10"/>
       <c r="S9" s="10"/>
@@ -31527,47 +31680,47 @@
     </row>
     <row r="10" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I10" s="11"/>
       <c r="J10" s="11"/>
       <c r="K10" s="11" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L10" s="11"/>
       <c r="M10" s="13" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="N10" s="11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O10" s="13" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="P10" s="11"/>
       <c r="Q10" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R10" s="11"/>
       <c r="S10" s="11"/>
@@ -31584,47 +31737,47 @@
     </row>
     <row r="11" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="H11" s="15" t="s">
         <v>141</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="G11" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="H11" s="15" t="s">
-        <v>144</v>
       </c>
       <c r="I11" s="14"/>
       <c r="J11" s="14"/>
       <c r="K11" s="14" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L11" s="14"/>
       <c r="M11" s="15" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="N11" s="14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O11" s="15" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="P11" s="14"/>
       <c r="Q11" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R11" s="14"/>
       <c r="S11" s="14"/>
@@ -31641,47 +31794,47 @@
     </row>
     <row r="12" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="I12" s="14"/>
       <c r="J12" s="14"/>
       <c r="K12" s="14" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L12" s="14"/>
       <c r="M12" s="15" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="N12" s="14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O12" s="15" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="P12" s="14"/>
       <c r="Q12" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R12" s="14"/>
       <c r="S12" s="14"/>
@@ -31698,47 +31851,47 @@
     </row>
     <row r="13" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C13" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I13" s="14"/>
       <c r="J13" s="14"/>
       <c r="K13" s="14" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L13" s="14"/>
       <c r="M13" s="15" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="N13" s="14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O13" s="15" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="P13" s="14"/>
       <c r="Q13" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R13" s="14"/>
       <c r="S13" s="14"/>
@@ -31755,47 +31908,47 @@
     </row>
     <row r="14" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C14" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I14" s="14"/>
       <c r="J14" s="14"/>
       <c r="K14" s="14" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L14" s="14"/>
       <c r="M14" s="15" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="N14" s="14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O14" s="15" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="P14" s="14"/>
       <c r="Q14" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R14" s="14"/>
       <c r="S14" s="14"/>
@@ -31812,47 +31965,47 @@
     </row>
     <row r="15" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C15" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I15" s="14"/>
       <c r="J15" s="14"/>
       <c r="K15" s="14" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L15" s="14"/>
       <c r="M15" s="15" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="N15" s="14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O15" s="15" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="P15" s="14"/>
       <c r="Q15" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R15" s="14"/>
       <c r="S15" s="14"/>
@@ -31869,47 +32022,47 @@
     </row>
     <row r="16" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C16" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I16" s="14"/>
       <c r="J16" s="14"/>
       <c r="K16" s="14" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L16" s="14"/>
       <c r="M16" s="15" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="N16" s="14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O16" s="15" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="P16" s="14"/>
       <c r="Q16" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R16" s="14"/>
       <c r="S16" s="14"/>
@@ -31926,192 +32079,192 @@
     </row>
     <row r="17" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F17" s="16" t="s">
+        <v>162</v>
+      </c>
+      <c r="G17" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="H17" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="J17" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="G17" s="16" t="s">
-        <v>166</v>
-      </c>
-      <c r="H17" s="17" t="s">
-        <v>167</v>
-      </c>
-      <c r="J17" s="16" t="s">
-        <v>168</v>
-      </c>
       <c r="K17" s="16" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L17" s="16" t="s">
         <v>22</v>
       </c>
       <c r="M17" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="N17" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="O17" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="Q17" s="3" t="s">
         <v>169</v>
-      </c>
-      <c r="N17" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="O17" s="17" t="s">
-        <v>171</v>
-      </c>
-      <c r="Q17" s="3" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="18" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H18" s="17" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J18" s="16" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K18" s="16" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L18" s="16" t="s">
         <v>22</v>
       </c>
       <c r="M18" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="N18" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="O18" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="Q18" s="3" t="s">
         <v>169</v>
-      </c>
-      <c r="N18" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="O18" s="17" t="s">
-        <v>171</v>
-      </c>
-      <c r="Q18" s="3" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="19" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="H19" s="17" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J19" s="16" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="K19" s="16" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L19" s="16" t="s">
         <v>22</v>
       </c>
       <c r="M19" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="N19" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="O19" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="Q19" s="3" t="s">
         <v>169</v>
-      </c>
-      <c r="N19" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="O19" s="17" t="s">
-        <v>171</v>
-      </c>
-      <c r="Q19" s="3" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="20" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>180</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="G20" s="18" t="s">
+        <v>181</v>
+      </c>
+      <c r="H20" s="18" t="s">
         <v>182</v>
-      </c>
-      <c r="B20" s="18" t="s">
-        <v>183</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D20" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>175</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>165</v>
-      </c>
-      <c r="G20" s="18" t="s">
-        <v>184</v>
-      </c>
-      <c r="H20" s="18" t="s">
-        <v>185</v>
       </c>
       <c r="I20" s="18"/>
       <c r="J20" s="18" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="K20" s="18" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L20" s="18" t="s">
         <v>22</v>
       </c>
       <c r="M20" s="19" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="N20" s="18" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O20" s="17" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="P20" s="18"/>
       <c r="Q20" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R20" s="18"/>
       <c r="S20" s="18"/>
@@ -32128,51 +32281,51 @@
     </row>
     <row r="21" spans="1:29" ht="87.5" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E21" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="F21" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="G21" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="H21" s="20" t="s">
         <v>190</v>
       </c>
-      <c r="F21" s="20" t="s">
+      <c r="I21" s="23" t="s">
         <v>191</v>
-      </c>
-      <c r="G21" s="22" t="s">
-        <v>192</v>
-      </c>
-      <c r="H21" s="20" t="s">
-        <v>193</v>
-      </c>
-      <c r="I21" s="23" t="s">
-        <v>194</v>
       </c>
       <c r="J21" s="24"/>
       <c r="K21" s="24" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L21" s="24"/>
       <c r="M21" s="25" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="N21" s="20" t="s">
         <v>24</v>
       </c>
       <c r="O21" s="21" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="P21" s="26" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="Q21" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R21" s="24"/>
       <c r="S21" s="24"/>
@@ -32189,237 +32342,237 @@
     </row>
     <row r="22" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="E22" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="F22" s="23" t="s">
         <v>198</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="G22" s="23" t="s">
         <v>199</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="E22" s="23" t="s">
+      <c r="H22" s="27" t="s">
         <v>200</v>
       </c>
-      <c r="F22" s="23" t="s">
+      <c r="I22" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="M22" s="17" t="s">
         <v>201</v>
       </c>
-      <c r="G22" s="23" t="s">
+      <c r="N22" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="O22" s="17" t="s">
         <v>202</v>
       </c>
-      <c r="H22" s="27" t="s">
-        <v>203</v>
-      </c>
-      <c r="I22" s="23" t="s">
+      <c r="P22" s="26" t="s">
         <v>194</v>
       </c>
-      <c r="K22" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="M22" s="17" t="s">
-        <v>204</v>
-      </c>
-      <c r="N22" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="O22" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="P22" s="26" t="s">
-        <v>197</v>
-      </c>
       <c r="Q22" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D23" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="E23" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="F23" s="28" t="s">
+        <v>205</v>
+      </c>
+      <c r="G23" s="23" t="s">
         <v>206</v>
       </c>
-      <c r="B23" s="16" t="s">
-        <v>207</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D23" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="E23" s="23" t="s">
+      <c r="H23" s="27" t="s">
         <v>200</v>
       </c>
-      <c r="F23" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="G23" s="23" t="s">
-        <v>209</v>
-      </c>
-      <c r="H23" s="27" t="s">
-        <v>203</v>
-      </c>
       <c r="I23" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="M23" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="N23" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="O23" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="P23" s="26" t="s">
         <v>194</v>
       </c>
-      <c r="K23" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="M23" s="17" t="s">
-        <v>204</v>
-      </c>
-      <c r="N23" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="O23" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="P23" s="26" t="s">
-        <v>197</v>
-      </c>
       <c r="Q23" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="24" spans="1:29" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D24" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="E24" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="F24" s="23" t="s">
         <v>210</v>
       </c>
-      <c r="B24" s="16" t="s">
+      <c r="G24" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D24" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="E24" s="23" t="s">
+      <c r="H24" s="27" t="s">
         <v>212</v>
       </c>
-      <c r="F24" s="23" t="s">
+      <c r="I24" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="M24" s="17" t="s">
         <v>213</v>
       </c>
-      <c r="G24" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="H24" s="27" t="s">
-        <v>215</v>
-      </c>
-      <c r="I24" s="23" t="s">
-        <v>194</v>
-      </c>
-      <c r="K24" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="M24" s="17" t="s">
-        <v>216</v>
-      </c>
       <c r="N24" s="16" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O24" s="17"/>
       <c r="P24" s="26" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="Q24" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="25" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>215</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="E25" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>216</v>
+      </c>
+      <c r="G25" s="16" t="s">
         <v>217</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="H25" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D25" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="E25" s="23" t="s">
-        <v>200</v>
-      </c>
-      <c r="F25" s="23" t="s">
+      <c r="I25" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="M25" s="17" t="s">
         <v>219</v>
       </c>
-      <c r="G25" s="16" t="s">
-        <v>220</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="I25" s="23" t="s">
+      <c r="N25" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="O25" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="P25" s="26" t="s">
         <v>194</v>
       </c>
-      <c r="K25" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="M25" s="17" t="s">
-        <v>222</v>
-      </c>
-      <c r="N25" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="O25" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="P25" s="26" t="s">
-        <v>197</v>
-      </c>
       <c r="Q25" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="26" spans="1:29" ht="75" x14ac:dyDescent="0.25">
       <c r="A26" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="E26" s="29" t="s">
+        <v>197</v>
+      </c>
+      <c r="F26" s="29" t="s">
+        <v>222</v>
+      </c>
+      <c r="G26" s="18" t="s">
         <v>223</v>
       </c>
-      <c r="B26" s="18" t="s">
-        <v>224</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D26" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="E26" s="29" t="s">
-        <v>200</v>
-      </c>
-      <c r="F26" s="29" t="s">
-        <v>225</v>
-      </c>
-      <c r="G26" s="18" t="s">
-        <v>226</v>
-      </c>
       <c r="H26" s="6" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="I26" s="23" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="J26" s="18"/>
       <c r="K26" s="18" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L26" s="18"/>
       <c r="M26" s="19" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="N26" s="18" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O26" s="19" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="P26" s="26" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R26" s="18"/>
       <c r="S26" s="18"/>
@@ -32436,336 +32589,336 @@
     </row>
     <row r="27" spans="1:29" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="B27" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E27" s="16" t="s">
         <v>227</v>
       </c>
-      <c r="B27" s="16" t="s">
+      <c r="F27" s="16" t="s">
         <v>228</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D27" s="16" t="s">
+      <c r="G27" s="16" t="s">
         <v>229</v>
       </c>
-      <c r="E27" s="16" t="s">
+      <c r="H27" s="17" t="s">
         <v>230</v>
       </c>
-      <c r="F27" s="16" t="s">
+      <c r="K27" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="M27" s="17" t="s">
         <v>231</v>
       </c>
-      <c r="G27" s="16" t="s">
+      <c r="N27" s="16" t="s">
         <v>232</v>
       </c>
-      <c r="H27" s="17" t="s">
+      <c r="O27" s="17" t="s">
         <v>233</v>
       </c>
-      <c r="K27" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="M27" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="N27" s="16" t="s">
-        <v>235</v>
-      </c>
-      <c r="O27" s="17" t="s">
-        <v>236</v>
-      </c>
       <c r="Q27" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="28" spans="1:29" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="F28" s="16" t="s">
         <v>237</v>
       </c>
-      <c r="B28" s="16" t="s">
+      <c r="G28" s="16" t="s">
         <v>238</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>229</v>
-      </c>
-      <c r="E28" s="16" t="s">
+      <c r="H28" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="F28" s="16" t="s">
+      <c r="K28" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="M28" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="N28" s="16" t="s">
+        <v>232</v>
+      </c>
+      <c r="O28" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="G28" s="16" t="s">
-        <v>241</v>
-      </c>
-      <c r="H28" s="17" t="s">
-        <v>242</v>
-      </c>
-      <c r="K28" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="M28" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="N28" s="16" t="s">
-        <v>235</v>
-      </c>
-      <c r="O28" s="17" t="s">
-        <v>243</v>
-      </c>
       <c r="Q28" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="29" spans="1:29" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="G29" s="16" t="s">
         <v>22</v>
       </c>
       <c r="H29" s="17" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="K29" s="16" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="M29" s="17" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="N29" s="16" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="O29" s="17" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="Q29" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="30" spans="1:29" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D30" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="E30" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="F30" s="16" t="s">
+        <v>251</v>
+      </c>
+      <c r="G30" s="16" t="s">
         <v>252</v>
       </c>
-      <c r="E30" s="16" t="s">
+      <c r="H30" s="27" t="s">
         <v>253</v>
       </c>
-      <c r="F30" s="16" t="s">
+      <c r="K30" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="M30" s="17" t="s">
         <v>254</v>
       </c>
-      <c r="G30" s="16" t="s">
+      <c r="O30" s="17" t="s">
         <v>255</v>
       </c>
-      <c r="H30" s="27" t="s">
-        <v>256</v>
-      </c>
-      <c r="K30" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="M30" s="17" t="s">
-        <v>257</v>
-      </c>
-      <c r="O30" s="17" t="s">
-        <v>258</v>
-      </c>
       <c r="Q30" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="31" spans="1:29" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="E31" s="16" t="s">
         <v>22</v>
       </c>
       <c r="F31" s="16" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="G31" s="16" t="s">
         <v>22</v>
       </c>
       <c r="H31" s="27" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="K31" s="16" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="M31" s="17" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="O31" s="17" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="Q31" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="32" spans="1:29" ht="50" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D32" s="16" t="s">
+        <v>262</v>
+      </c>
+      <c r="E32" s="16" t="s">
+        <v>263</v>
+      </c>
+      <c r="F32" s="16" t="s">
+        <v>264</v>
+      </c>
+      <c r="G32" s="16" t="s">
         <v>265</v>
       </c>
-      <c r="E32" s="16" t="s">
+      <c r="H32" s="27" t="s">
         <v>266</v>
       </c>
-      <c r="F32" s="16" t="s">
-        <v>267</v>
-      </c>
-      <c r="G32" s="16" t="s">
-        <v>268</v>
-      </c>
-      <c r="H32" s="27" t="s">
-        <v>269</v>
-      </c>
       <c r="I32" s="30" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="J32" s="16" t="s">
         <v>22</v>
       </c>
       <c r="K32" s="16" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="M32" s="17" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="O32" s="17" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="Q32" s="3" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="33" spans="1:29" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="16" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D33" s="16" t="s">
+        <v>270</v>
+      </c>
+      <c r="E33" s="16" t="s">
+        <v>271</v>
+      </c>
+      <c r="F33" s="16" t="s">
+        <v>272</v>
+      </c>
+      <c r="G33" s="31" t="s">
         <v>273</v>
       </c>
-      <c r="E33" s="16" t="s">
+      <c r="H33" s="27" t="s">
         <v>274</v>
       </c>
-      <c r="F33" s="16" t="s">
+      <c r="J33" s="16" t="s">
         <v>275</v>
       </c>
-      <c r="G33" s="31" t="s">
+      <c r="K33" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="M33" s="17" t="s">
         <v>276</v>
       </c>
-      <c r="H33" s="27" t="s">
+      <c r="N33" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="O33" s="17" t="s">
         <v>277</v>
       </c>
-      <c r="J33" s="16" t="s">
-        <v>278</v>
-      </c>
-      <c r="K33" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="M33" s="17" t="s">
-        <v>279</v>
-      </c>
-      <c r="N33" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="O33" s="17" t="s">
-        <v>280</v>
-      </c>
       <c r="Q33" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:29" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="32" t="s">
+        <v>278</v>
+      </c>
+      <c r="B34" s="16" t="s">
+        <v>279</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="E34" s="32" t="s">
+        <v>280</v>
+      </c>
+      <c r="F34" s="32" t="s">
         <v>281</v>
       </c>
-      <c r="B34" s="16" t="s">
+      <c r="G34" s="32" t="s">
         <v>282</v>
       </c>
-      <c r="C34" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D34" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="E34" s="32" t="s">
+      <c r="H34" s="33" t="s">
         <v>283</v>
-      </c>
-      <c r="F34" s="32" t="s">
-        <v>284</v>
-      </c>
-      <c r="G34" s="32" t="s">
-        <v>285</v>
-      </c>
-      <c r="H34" s="33" t="s">
-        <v>286</v>
       </c>
       <c r="I34" s="32"/>
       <c r="J34" s="32" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="K34" s="16" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L34" s="32"/>
       <c r="M34" s="34" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="N34" s="32" t="s">
         <v>24</v>
       </c>
       <c r="O34" s="33" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="P34" s="32"/>
       <c r="Q34" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R34" s="32"/>
       <c r="S34" s="32"/>
@@ -32782,49 +32935,49 @@
     </row>
     <row r="35" spans="1:29" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="32" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E35" s="32" t="s">
+        <v>280</v>
+      </c>
+      <c r="F35" s="32" t="s">
+        <v>281</v>
+      </c>
+      <c r="G35" s="32" t="s">
+        <v>288</v>
+      </c>
+      <c r="H35" s="33" t="s">
         <v>283</v>
-      </c>
-      <c r="F35" s="32" t="s">
-        <v>284</v>
-      </c>
-      <c r="G35" s="32" t="s">
-        <v>291</v>
-      </c>
-      <c r="H35" s="33" t="s">
-        <v>286</v>
       </c>
       <c r="I35" s="32"/>
       <c r="J35" s="32" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="K35" s="16" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L35" s="32"/>
       <c r="M35" s="34" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="N35" s="32" t="s">
         <v>24</v>
       </c>
       <c r="O35" s="33" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="P35" s="32"/>
       <c r="Q35" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R35" s="32"/>
       <c r="S35" s="32"/>
@@ -32841,93 +32994,93 @@
     </row>
     <row r="36" spans="1:29" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E36" s="35" t="s">
+        <v>291</v>
+      </c>
+      <c r="F36" s="16" t="s">
+        <v>292</v>
+      </c>
+      <c r="G36" s="16" t="s">
+        <v>293</v>
+      </c>
+      <c r="H36" s="17" t="s">
         <v>294</v>
       </c>
-      <c r="F36" s="16" t="s">
+      <c r="J36" s="16" t="s">
+        <v>275</v>
+      </c>
+      <c r="K36" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="M36" s="31" t="s">
         <v>295</v>
-      </c>
-      <c r="G36" s="16" t="s">
-        <v>296</v>
-      </c>
-      <c r="H36" s="17" t="s">
-        <v>297</v>
-      </c>
-      <c r="J36" s="16" t="s">
-        <v>278</v>
-      </c>
-      <c r="K36" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="M36" s="31" t="s">
-        <v>298</v>
       </c>
       <c r="N36" s="16" t="s">
         <v>24</v>
       </c>
       <c r="O36" s="17" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="37" spans="1:29" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A37" s="32" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B37" s="32" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D37" s="32" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E37" s="30" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="F37" s="32" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="G37" s="32" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="H37" s="36" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="I37" s="32"/>
       <c r="J37" s="32" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="K37" s="16" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L37" s="32"/>
       <c r="M37" s="34" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="N37" s="32" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O37" s="33" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="P37" s="32"/>
       <c r="Q37" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R37" s="32"/>
       <c r="S37" s="32"/>
@@ -32944,49 +33097,49 @@
     </row>
     <row r="38" spans="1:29" ht="87.5" x14ac:dyDescent="0.25">
       <c r="A38" s="32" t="s">
+        <v>302</v>
+      </c>
+      <c r="B38" s="32" t="s">
+        <v>303</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D38" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="E38" s="30" t="s">
+        <v>271</v>
+      </c>
+      <c r="F38" s="32" t="s">
+        <v>304</v>
+      </c>
+      <c r="G38" s="32" t="s">
         <v>305</v>
       </c>
-      <c r="B38" s="32" t="s">
-        <v>306</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D38" s="32" t="s">
-        <v>83</v>
-      </c>
-      <c r="E38" s="30" t="s">
+      <c r="H38" s="36" t="s">
         <v>274</v>
-      </c>
-      <c r="F38" s="32" t="s">
-        <v>307</v>
-      </c>
-      <c r="G38" s="32" t="s">
-        <v>308</v>
-      </c>
-      <c r="H38" s="36" t="s">
-        <v>277</v>
       </c>
       <c r="I38" s="32"/>
       <c r="J38" s="32" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="K38" s="32" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L38" s="32"/>
       <c r="M38" s="34" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="N38" s="32" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O38" s="33" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="P38" s="32"/>
       <c r="Q38" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="R38" s="32"/>
       <c r="S38" s="32"/>

</xml_diff>